<commit_message>
cambios en el prompt
</commit_message>
<xml_diff>
--- a/src/output.xlsx
+++ b/src/output.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -415,39 +415,87 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>Body Lily-Negro-S</v>
+        <v>Short Cloe-Terracotta-S</v>
       </c>
       <c r="B2" t="str">
-        <v>Aumenta el glamour al vestir este body lily negro, diseñado para realzar tus figuras y ofrecer una silueta ajustada con un decollete triangular y caderas en forma de V. Combina estilo y comodidad para lucir perfecto en cualquier evento, dejando tu modernidad y elegancia al descubierto.</v>
+        <v>Nuestro armario es la solución perfecta para convertir tus días en momentos de relajación y agregar un toque chic a tu estilo.</v>
       </c>
       <c r="C2" t="str" xml:space="preserve">
-        <v xml:space="preserve">Ajustado para realzar tus curvas
-Triángulo del decollete en el pecho
-Caderas en forma de V para una silueta dinámica</v>
+        <v xml:space="preserve">Dimensiones acogedoras para un espacio cómodo y elegante
+Color terracota suave para una apariencia sofisticada
+Boca de armario con cerradura para seguridad</v>
       </c>
       <c r="D2" t="str">
-        <v>&lt;body&gt;&lt;ul&gt;&lt;li&gt;Deslumbra con elegancia&lt;/li&gt;&lt;li&gt;Diseñado con silueta ajustada&lt;/li&gt;&lt;li&gt;Favorece escote triangular&lt;/li&gt;&lt;li&gt;Cargaderas en forma de V&lt;/li&gt;&lt;li&gt;Combina estilo y comodidad&lt;/li&gt;&lt;li&gt;Ideal para destacar en cualquier ocasión&lt;/li&gt;&lt;li&gt;Ofrece un toque de sofisticación y modernidad&lt;/li&gt;&lt;/ul&gt;&lt;/body&gt;</v>
+        <v>&lt;body&gt;&lt;h2&gt;Short Cloe-Terracotta-S&lt;/h2&gt;&lt;p&gt;Nuestro armario es el complemento ideal para disfrutar cómodamente tus días y agregar un toque chic a tu apariencia.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Diseñado con dimensiones acogedoras para maximizar el espacio.&lt;/li&gt;&lt;li&gt;Color terracota suave proporciona una apariencia sofisticada.&lt;/li&gt;&lt;li&gt;Boca de armario cerradura asegurando la seguridad de tus pertenencias.&lt;/li&gt;&lt;/ul&gt;&lt;/body&gt;</v>
       </c>
     </row>
     <row r="3" xml:space="preserve">
       <c r="A3" t="str">
-        <v>Vestido Largo Reverie-Negro-L</v>
+        <v>Short Cloe-Terracotta XS</v>
       </c>
       <c r="B3" t="str">
-        <v>Explorar la elegancia con nuestro Vestido de Talle Medio Revelación, con una silueta ligeramente ajustada, un cuello profundo en V decorado con tiras cruzadas en la cintura, mangas largas y una falda seductora con una apertura en el frente. Asegura el estilo con este diseño único y encantador.</v>
+        <v>Un armario compacto y funcional que combina comodidad y estilo para completar tu look diario.</v>
       </c>
       <c r="C3" t="str" xml:space="preserve">
-        <v xml:space="preserve">Vestido de talle medio semi ajustado
-Cuello profundo V adornado con tiras cruzadas
-Mangas largas y falda seductora con apertura en frente</v>
+        <v xml:space="preserve">Dimensiones prácticas para un espacio limitado
+Materiales suaves y duraderos para mayor comodidad
+Color terracota y diseño Cloe para una apariencia sofisticada</v>
       </c>
       <c r="D3" t="str">
-        <v>&lt;body&gt;&lt;h1&gt;Vestido Largo Revelación&lt;/h1&gt;&lt;p&gt;Un vestido de talle medio semi ajustado, cuello profundo en V con tiras cruzadas en la cintura, mangas largas y una falda seductora con apertura en frente. Encuentra el estilo perfecto con este diseño único y cautivador.&lt;/p&gt;&lt;/body&gt;</v>
+        <v>&lt;body&gt;&lt;h2&gt;Short Cloe-Terracotta XS&lt;/h2&gt;&lt;p&gt;Un armario compacto diseñado para complementar tu estilo diario. Con materiales suaves y duraderos, este armario práctico se adapta perfectamente a espacios limitados. Su color terracota y diseño Cloe le dan un toque sofisticado y fashionable.&lt;/p&gt;&lt;/body&gt;</v>
+      </c>
+    </row>
+    <row r="4" xml:space="preserve">
+      <c r="A4" t="str">
+        <v>Short Cloe-Terracotta-L</v>
+      </c>
+      <c r="B4" t="str">
+        <v>El armario Short Cloe-Terracota-L es la solución ideal para agregar cómoda y elegancia a tu espacio de vestuario. Con una silueta ajustada que realza tus curvas, un escote cruzado en el frente para una apariencia más voluminosa, y cargaderas ajustables para mayor comodidad, este armario te ofrece un look sofisticado y funcional.</v>
+      </c>
+      <c r="C4" t="str" xml:space="preserve">
+        <v xml:space="preserve">Silueta ajustada: Realza tus curvas para un aspecto encantador
+Escote cruzado en el frente: Agrega volumen y elegancia a tu figura
+Cargaderas ajustables: Acomoda perfectamente a tu cuerpo</v>
+      </c>
+      <c r="D4" t="str">
+        <v>&lt;body&gt;&lt;h2&gt;Short Cloe-Terracotta-L&lt;/h2&gt;&lt;p&gt;El armario Short Cloe-Terracota-L es el complemento perfecto para llenar tus días de comodidad y un toque fashionista. Con una silueta ajustada que realza tus curvas, un escote cruzado en el frente para una apariencia más voluminosa, y cargaderas ajustables para mayor comodidad, este armario te ofrece un look sofisticado y funcional.&lt;/p&gt;&lt;/body&gt;</v>
+      </c>
+    </row>
+    <row r="5" xml:space="preserve">
+      <c r="A5" t="str">
+        <v>Vestido Largo Aires Del Norte-Memory_Mul</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Mejorarlo tomando en cuenta la data suministrada</v>
+      </c>
+      <c r="C5" t="str" xml:space="preserve">
+        <v xml:space="preserve">Silueta ajustada que realza las curvas
+Escote semi-curvo con jareta para un toque bohemio
+Cut out laterales para un toque moderno y seductor</v>
+      </c>
+      <c r="D5" t="str">
+        <v>&lt;body&gt;&lt;h2&gt;Vestido Largo Aires Del Norte-Memory_Mul&lt;/h2&gt;&lt;br/&gt;&lt;p style="text-align:justify"&gt;&lt;span style="font-size:18px"&gt;Este vestido largo fusiona la moda con detalles únicos, creando una pieza esencial para destacar con estilo en cualquier ocasión.&lt;/span&gt;&lt;/p&gt;&lt;br/&gt;&lt;p style="font-size:18px"&gt;&lt;strong&gt;Destacado&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li style="font-size:16px"&gt;Silueta ajustada que realza las curvas&lt;/li&gt;&lt;li style="font-size:16px"&gt;Escote semi-curvo con jareta para un toque bohemio&lt;/li&gt;&lt;li style="font-size:16px"&gt;Cut out laterales para un toque moderno y seductor&lt;/li&gt;&lt;/ul&gt;&lt;/body&gt;</v>
+      </c>
+    </row>
+    <row r="6" xml:space="preserve">
+      <c r="A6" t="str">
+        <v>Camisa Alexa-Estampado Verde-M</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Mejorarlo tomando en cuenta la data suministrada</v>
+      </c>
+      <c r="C6" t="str" xml:space="preserve">
+        <v xml:space="preserve">Descripción corta del punto 1
+Descripción corta del punto 2
+Descripción corta del punto 3</v>
+      </c>
+      <c r="D6" t="str">
+        <v>&lt;body&gt;...&lt;/body&gt;</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>